<commit_message>
Cambio de la perspectiva del TFG
Tras realizar una reunión con el tutor, no se ha visto viable la línea de desarrollo del TFG, por lo que se ha modificado la perspectiva final, así como su alcance.
</commit_message>
<xml_diff>
--- a/datos/ListaExcel/ListaPersonas1.xlsx
+++ b/datos/ListaExcel/ListaPersonas1.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universidaddeburgos-my.sharepoint.com/personal/mmm1059_alu_ubu_es/Documents/Escritorio/TFG-Marina-Martin/datos/ListaExcel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="193" documentId="8_{1358C022-85BE-4B7F-BF4E-FCC1DD1B9E1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6FA6B87B-CE25-44A0-9729-DAA8F01C110D}"/>
+  <xr:revisionPtr revIDLastSave="196" documentId="8_{1358C022-85BE-4B7F-BF4E-FCC1DD1B9E1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2761EEFA-EDC9-4F4C-872B-3C2C496CD890}"/>
   <bookViews>
-    <workbookView xWindow="924" yWindow="1176" windowWidth="10164" windowHeight="9780" xr2:uid="{B0B6A5FC-CE1B-471C-8D49-49C1E4593AB9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B0B6A5FC-CE1B-471C-8D49-49C1E4593AB9}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="2" r:id="rId1"/>
     <sheet name="HojaN" sheetId="1" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcCompleted="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -457,6 +457,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1740,9 +1744,18 @@
       <c r="B35" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F35" s="3" t="e">
+      <c r="C35">
+        <v>21</v>
+      </c>
+      <c r="D35">
+        <v>80</v>
+      </c>
+      <c r="E35">
+        <v>1.74</v>
+      </c>
+      <c r="F35" s="3">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
+        <v>26.423569824283259</v>
       </c>
       <c r="G35" t="s">
         <v>35</v>

</xml_diff>